<commit_message>
fix:updated attributes for cancel on_cancel
</commit_message>
<xml_diff>
--- a/Attribute_List_Motor(2026).xlsx
+++ b/Attribute_List_Motor(2026).xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7057" uniqueCount="628">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7057" uniqueCount="630">
   <si>
     <t>Path</t>
   </si>
@@ -1967,6 +1967,9 @@
     </r>
   </si>
   <si>
+    <t>cancel</t>
+  </si>
+  <si>
     <t>message.cancellation_reason_id</t>
   </si>
   <si>
@@ -1986,6 +1989,9 @@
   </si>
   <si>
     <t>This refers to the description of the descriptor object</t>
+  </si>
+  <si>
+    <t>on_cancel</t>
   </si>
   <si>
     <t>CANCELLATION_INITIATED</t>
@@ -24824,8 +24830,8 @@
       <c r="D10" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E10" s="1" t="s">
-        <v>597</v>
+      <c r="E10" s="55" t="s">
+        <v>619</v>
       </c>
       <c r="F10" s="3" t="s">
         <v>36</v>
@@ -24933,7 +24939,7 @@
     </row>
     <row r="16">
       <c r="A16" s="55" t="s">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="B16" s="18" t="s">
         <v>52</v>
@@ -24948,12 +24954,12 @@
         <v>5.0</v>
       </c>
       <c r="F16" s="57" t="s">
-        <v>620</v>
+        <v>621</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="58" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="B17" s="18" t="s">
         <v>52</v>
@@ -24965,10 +24971,10 @@
         <v>9</v>
       </c>
       <c r="E17" s="58" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="F17" s="57" t="s">
-        <v>623</v>
+        <v>624</v>
       </c>
     </row>
     <row r="18">
@@ -25033,7 +25039,7 @@
     </row>
     <row r="21">
       <c r="A21" s="59" t="s">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="B21" s="30" t="s">
         <v>52</v>
@@ -25048,7 +25054,7 @@
         <v>74</v>
       </c>
       <c r="F21" s="60" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
     </row>
   </sheetData>
@@ -25269,8 +25275,8 @@
       <c r="D10" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E10" s="1" t="s">
-        <v>557</v>
+      <c r="E10" s="55" t="s">
+        <v>627</v>
       </c>
       <c r="F10" s="3" t="s">
         <v>36</v>
@@ -26190,7 +26196,7 @@
         <v>45</v>
       </c>
       <c r="E56" s="55" t="s">
-        <v>626</v>
+        <v>628</v>
       </c>
       <c r="F56" s="1" t="s">
         <v>568</v>
@@ -26938,7 +26944,7 @@
     </row>
     <row r="94">
       <c r="A94" s="1" t="s">
-        <v>627</v>
+        <v>629</v>
       </c>
       <c r="B94" s="18" t="s">
         <v>44</v>

</xml_diff>